<commit_message>
rfq reply as xlsx attachment now extracts the prices
</commit_message>
<xml_diff>
--- a/data/supplier_catalog.xlsx
+++ b/data/supplier_catalog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marika.ivanova\PycharmProjects\AIPurchaseAssistant\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A016B7-7AA7-4E22-902C-8C7644C8FD10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DFBF549-F7A1-4CF8-B217-1FD713E0F4CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="190">
   <si>
     <t>ARHAM INTERNATIONAL GEMS</t>
   </si>
@@ -759,6 +759,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -771,7 +772,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1080,102 +1080,102 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:93" ht="18" x14ac:dyDescent="0.4">
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="10"/>
-      <c r="T1" s="8" t="s">
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="11"/>
+      <c r="T1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9"/>
-      <c r="W1" s="9"/>
-      <c r="X1" s="9"/>
-      <c r="Y1" s="9"/>
-      <c r="Z1" s="9"/>
-      <c r="AA1" s="9"/>
-      <c r="AB1" s="9"/>
-      <c r="AC1" s="9"/>
-      <c r="AD1" s="9"/>
-      <c r="AE1" s="9"/>
-      <c r="AF1" s="9"/>
-      <c r="AG1" s="9"/>
-      <c r="AH1" s="9"/>
-      <c r="AI1" s="9"/>
-      <c r="AJ1" s="9"/>
-      <c r="AK1" s="9"/>
-      <c r="AL1" s="9"/>
-      <c r="AM1" s="9"/>
-      <c r="AN1" s="9"/>
-      <c r="AO1" s="9"/>
-      <c r="AP1" s="9"/>
-      <c r="AQ1" s="9"/>
-      <c r="AR1" s="9"/>
-      <c r="AS1" s="9"/>
-      <c r="AT1" s="9"/>
-      <c r="AU1" s="9"/>
-      <c r="AV1" s="9"/>
-      <c r="AW1" s="9"/>
-      <c r="AX1" s="9"/>
-      <c r="AY1" s="9"/>
-      <c r="AZ1" s="9"/>
-      <c r="BA1" s="9"/>
-      <c r="BB1" s="9"/>
-      <c r="BC1" s="9"/>
-      <c r="BD1" s="9"/>
-      <c r="BE1" s="9"/>
-      <c r="BF1" s="9"/>
-      <c r="BG1" s="9"/>
-      <c r="BH1" s="9"/>
-      <c r="BI1" s="9"/>
-      <c r="BJ1" s="9"/>
-      <c r="BK1" s="9"/>
-      <c r="BL1" s="9"/>
-      <c r="BM1" s="9"/>
-      <c r="BN1" s="9"/>
-      <c r="BO1" s="9"/>
-      <c r="BP1" s="9"/>
-      <c r="BQ1" s="9"/>
-      <c r="BR1" s="9"/>
-      <c r="BS1" s="9"/>
-      <c r="BT1" s="9"/>
-      <c r="BU1" s="9"/>
-      <c r="BV1" s="9"/>
-      <c r="BW1" s="9"/>
-      <c r="BX1" s="9"/>
-      <c r="BY1" s="9"/>
-      <c r="BZ1" s="9"/>
-      <c r="CA1" s="9"/>
-      <c r="CB1" s="9"/>
-      <c r="CC1" s="9"/>
-      <c r="CD1" s="9"/>
-      <c r="CE1" s="9"/>
-      <c r="CF1" s="9"/>
-      <c r="CG1" s="9"/>
-      <c r="CH1" s="9"/>
-      <c r="CI1" s="9"/>
-      <c r="CJ1" s="10"/>
-      <c r="CK1" s="7" t="s">
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
+      <c r="Y1" s="10"/>
+      <c r="Z1" s="10"/>
+      <c r="AA1" s="10"/>
+      <c r="AB1" s="10"/>
+      <c r="AC1" s="10"/>
+      <c r="AD1" s="10"/>
+      <c r="AE1" s="10"/>
+      <c r="AF1" s="10"/>
+      <c r="AG1" s="10"/>
+      <c r="AH1" s="10"/>
+      <c r="AI1" s="10"/>
+      <c r="AJ1" s="10"/>
+      <c r="AK1" s="10"/>
+      <c r="AL1" s="10"/>
+      <c r="AM1" s="10"/>
+      <c r="AN1" s="10"/>
+      <c r="AO1" s="10"/>
+      <c r="AP1" s="10"/>
+      <c r="AQ1" s="10"/>
+      <c r="AR1" s="10"/>
+      <c r="AS1" s="10"/>
+      <c r="AT1" s="10"/>
+      <c r="AU1" s="10"/>
+      <c r="AV1" s="10"/>
+      <c r="AW1" s="10"/>
+      <c r="AX1" s="10"/>
+      <c r="AY1" s="10"/>
+      <c r="AZ1" s="10"/>
+      <c r="BA1" s="10"/>
+      <c r="BB1" s="10"/>
+      <c r="BC1" s="10"/>
+      <c r="BD1" s="10"/>
+      <c r="BE1" s="10"/>
+      <c r="BF1" s="10"/>
+      <c r="BG1" s="10"/>
+      <c r="BH1" s="10"/>
+      <c r="BI1" s="10"/>
+      <c r="BJ1" s="10"/>
+      <c r="BK1" s="10"/>
+      <c r="BL1" s="10"/>
+      <c r="BM1" s="10"/>
+      <c r="BN1" s="10"/>
+      <c r="BO1" s="10"/>
+      <c r="BP1" s="10"/>
+      <c r="BQ1" s="10"/>
+      <c r="BR1" s="10"/>
+      <c r="BS1" s="10"/>
+      <c r="BT1" s="10"/>
+      <c r="BU1" s="10"/>
+      <c r="BV1" s="10"/>
+      <c r="BW1" s="10"/>
+      <c r="BX1" s="10"/>
+      <c r="BY1" s="10"/>
+      <c r="BZ1" s="10"/>
+      <c r="CA1" s="10"/>
+      <c r="CB1" s="10"/>
+      <c r="CC1" s="10"/>
+      <c r="CD1" s="10"/>
+      <c r="CE1" s="10"/>
+      <c r="CF1" s="10"/>
+      <c r="CG1" s="10"/>
+      <c r="CH1" s="10"/>
+      <c r="CI1" s="10"/>
+      <c r="CJ1" s="11"/>
+      <c r="CK1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="CL1" s="7"/>
-      <c r="CM1" s="7"/>
-      <c r="CN1" s="7"/>
+      <c r="CL1" s="8"/>
+      <c r="CM1" s="8"/>
+      <c r="CN1" s="8"/>
     </row>
     <row r="2" spans="2:93" ht="174.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
@@ -9422,7 +9422,9 @@
       <c r="AN78" s="6"/>
       <c r="AO78" s="6"/>
       <c r="AP78" s="6"/>
-      <c r="AQ78" s="6"/>
+      <c r="AQ78" s="6" t="s">
+        <v>167</v>
+      </c>
       <c r="AR78" s="6"/>
       <c r="AS78" s="6"/>
       <c r="AT78" s="6"/>
@@ -9446,7 +9448,9 @@
       <c r="BL78" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="BM78" s="6"/>
+      <c r="BM78" s="6" t="s">
+        <v>167</v>
+      </c>
       <c r="BN78" s="6"/>
       <c r="BO78" s="6" t="s">
         <v>167</v>
@@ -35205,7 +35209,7 @@
       <c r="C77" t="s">
         <v>187</v>
       </c>
-      <c r="D77" s="11" t="s">
+      <c r="D77" s="7" t="s">
         <v>188</v>
       </c>
     </row>
@@ -35216,7 +35220,7 @@
       <c r="C78" t="s">
         <v>187</v>
       </c>
-      <c r="D78" s="11" t="s">
+      <c r="D78" s="7" t="s">
         <v>189</v>
       </c>
     </row>

</xml_diff>